<commit_message>
docs: use display name in project documents
</commit_message>
<xml_diff>
--- a/deliverables/project-initiation/04-工业路由器装配MES-项目管理台账.xlsx
+++ b/deliverables/project-initiation/04-工业路由器装配MES-项目管理台账.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="R7b61f34bc18f4a02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求清单" sheetId="2" r:id="R8fe1d215ca1b48b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求追踪" sheetId="3" r:id="Rfda2a5f5c5974417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fit-Gap" sheetId="4" r:id="R8932ab9eea6e47ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RACI" sheetId="5" r:id="R6dc5e2dc791f4dc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="6" r:id="R1d9c71b12f6b4e03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAID" sheetId="7" r:id="Rbce4cce3384f40b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="接口清单" sheetId="8" r:id="Rf5cc62f336324c43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAT" sheetId="9" r:id="Rcd2ff529e83746a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待澄清问题" sheetId="10" r:id="Rb5d74470cf6749a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="Rb27a4927dcea4a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求清单" sheetId="2" r:id="R0c0b952df5b5432f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求追踪" sheetId="3" r:id="R5b5e24f388ab451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fit-Gap" sheetId="4" r:id="Rd9c7432f63f54fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RACI" sheetId="5" r:id="R2720afa61b244a75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="6" r:id="Ra87a8e5879484e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAID" sheetId="7" r:id="R128f11689ba2440d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="接口清单" sheetId="8" r:id="Ra3ca347d35fd4b59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAT" sheetId="9" r:id="Re97641a1a77149ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待澄清问题" sheetId="10" r:id="R8a88e26bc7b14170"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -562,7 +562,7 @@
         <x:v>负责人</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>李文韬</x:v>
+        <x:v>李先生</x:v>
       </x:c>
       <x:c r="D5" s="7" t="str">
         <x:v>需求总数</x:v>
@@ -951,7 +951,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37754da2a40d4703"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d30eb8b06764f36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2757,7 +2757,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a5a708461d64577"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02048dd2580847b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4223,7 +4223,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb35ea88a67648c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf90805ef977438d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4613,7 +4613,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97b74ca575a847b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4187ffbd80bf4445"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5003,7 +5003,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1ae91ab3ee74b8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree582322a2434c02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5588,7 +5588,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15786359e9a54b62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra397ce77fa1f4ed4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5962,7 +5962,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1cd097f50924489"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b120b2603b4d32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6232,7 +6232,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb60087c289044393"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bc81b4d76e54ff0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6366,7 +6366,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14bef17f6a3c4f9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd65f95f5f2384181"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>